<commit_message>
Add G6 Barcelona as Mexico in Group B (14 BSC teams total)
Mexico flips from a challenge team to a real BSC team (G6 Barcelona),
bringing Group B to 4 BSC teams with no challenge — matching Group D's
structure. Total field grows from 13 to 14.

- Added team id 14 (G6 Barcelona, Mexico, 6th, Girls) to all three apps
- GROUPS.B: [4,5,6] -> [4,5,6,14]
- Removed CHALLENGE_COUNTRIES.B
- Converted Group B's three weekly challenge matches (vs Mexico) into
  group matches between BSC teams 4/5/6 and 14
- Updated all "13 BSC" copy to "14 BSC" (announcements, How It Works,
  Challenge Teams card, At a Glance tile, All Teams header, scoring
  title placeholder, JS comments)
- "Groups A, B, C have challenges" -> "Groups A and C"
- Added G6 Barcelona row to scoresheet.xlsx (week 1 tab)
- CLAUDE.md updated with new group structure and team count

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoresheet.xlsx
+++ b/scoresheet.xlsx
@@ -1,103 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robschoen/Dropbox/CC/worldcup/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D9F568C-245E-3240-9E32-E2FFCF962822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="23160" yWindow="7480" windowWidth="27760" windowHeight="16680" xr2:uid="{E248547C-94F2-B54C-8B6E-5F8BCA1B34EC}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="23160" yWindow="7480" windowWidth="27760" windowHeight="16680" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="week 1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="week 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>B3 Atalanta</t>
-  </si>
-  <si>
-    <t>B3 Ipswich</t>
-  </si>
-  <si>
-    <t>G4 Reign</t>
-  </si>
-  <si>
-    <t>B4 Brentford</t>
-  </si>
-  <si>
-    <t>G5 Angel City</t>
-  </si>
-  <si>
-    <t>B5 Benfica</t>
-  </si>
-  <si>
-    <t>B5 Dortmund</t>
-  </si>
-  <si>
-    <t>B5 Napoli</t>
-  </si>
-  <si>
-    <t>G6 Arsenal</t>
-  </si>
-  <si>
-    <t>G7 Ajax</t>
-  </si>
-  <si>
-    <t>G7 Chelsea</t>
-  </si>
-  <si>
-    <t>G8 Courage</t>
-  </si>
-  <si>
-    <t>G8 Pride</t>
-  </si>
-  <si>
-    <t>Goals</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
       <name val="AndaleMono"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -116,21 +45,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -449,104 +437,121 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{E08B6DF5-7311-2F4A-9EA0-E96BACB9BBE1}">
-  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;fc6a4b13-d0ff-46f3-96f5-f4c198c43beb&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A196B1BD-25D2-4A4C-864B-A627E6A45B37}">
-  <dimension ref="A1:B14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="18.875" customWidth="1"/>
+    <col width="18.875" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="B1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
-        <v>12</v>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Goals</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B3 Atalanta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B3 Ipswich</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>G4 Reign</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B4 Brentford</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>G5 Angel City</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B5 Benfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B5 Dortmund</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B5 Napoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>G6 Arsenal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>G6 Barcelona</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>G7 Ajax</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>G7 Chelsea</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>G8 Courage</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>G8 Pride</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Process Week 1 results (Apr 27)
Records the 8 Week 1 matches in RESULTS across all three apps and
fills in scoresheet.xlsx for the record. Bumps CURRENT_WEEK to 2 in
the player and admin apps so the home countdown points to Matchday 2
on May 4. Coach app stays at Week 1 until Week 2 instructions arrive.

Notable outcomes (Group A: Reign 0 pts after losing to USA challenge;
Group B: Arsenal/Barcelona both win their openers; Group C: Pride
opens with 5-1 over Chelsea; Group D: Benfica and Courage take 3 pts).

Challenge teams (USA, Senegal) auto-compute to 4 (rounded avg of 14
BSC goals = 52/14 = 3.71).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoresheet.xlsx
+++ b/scoresheet.xlsx
@@ -462,6 +462,9 @@
           <t>B3 Atalanta</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -469,6 +472,9 @@
           <t>B3 Ipswich</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -476,6 +482,9 @@
           <t>G4 Reign</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -483,6 +492,9 @@
           <t>B4 Brentford</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -490,6 +502,9 @@
           <t>G5 Angel City</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -497,6 +512,9 @@
           <t>B5 Benfica</t>
         </is>
       </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -504,6 +522,9 @@
           <t>B5 Dortmund</t>
         </is>
       </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -511,6 +532,9 @@
           <t>B5 Napoli</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -518,6 +542,9 @@
           <t>G6 Arsenal</t>
         </is>
       </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -525,6 +552,9 @@
           <t>G6 Barcelona</t>
         </is>
       </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -532,6 +562,9 @@
           <t>G7 Ajax</t>
         </is>
       </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -539,6 +572,9 @@
           <t>G7 Chelsea</t>
         </is>
       </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -546,12 +582,18 @@
           <t>G8 Courage</t>
         </is>
       </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>G8 Pride</t>
         </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Roll coach app to Week 2 (May 4)
Replaces Week 1 trivia with Week 2's set:
- Q1: South American host of the 1930 men's World Cup (Uruguay)
- Q2: Chinese host city of the 1991 women's World Cup (Guangzhou)
- Q3: Country with most men's World Cup hostings after 2026 (Mexico)
- Q4: Name of the dog that found the stolen 1966 trophy (Pickles)
- Q5: Toe taps in 1 min (head-to-head, +1 goal to higher count)
- Hint: Week 3 will be juggling

CURRENT_WEEK bumped to 2. Adds the empty week 2 tab to scoresheet.xlsx
for Cathleen to fill after this Saturday's 6 PM deadline.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoresheet.xlsx
+++ b/scoresheet.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="week 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="week 2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -599,4 +600,126 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col width="18.875" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Goals</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B3 Atalanta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B3 Ipswich</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>G4 Reign</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B4 Brentford</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>G5 Angel City</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B5 Benfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B5 Dortmund</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B5 Napoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>G6 Arsenal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>G6 Barcelona</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>G7 Ajax</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>G7 Chelsea</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>G8 Courage</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>G8 Pride</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Process Week 2 results (May 4)
Records the 8 Week 2 matches in RESULTS across all three apps and
adds the week 2 tab to scoresheet.xlsx. Bumps CURRENT_WEEK to 3 in
the player and admin apps so the home countdown points to Matchday 3
on May 11.

Standings after Week 2:
- Group A: Angel City 4 pts, Ipswich 1, Reign 0
- Group B: Arsenal 4, Ajax + Barcelona 3, Dortmund 1
- Group C: Pride 6 (undefeated), Atalanta 4, Chelsea 0
- Group D: Courage 6 (undefeated), Benfica + Brentford 3, Napoli 0

Challenge teams (USA, Senegal) compute to 3 (40/14 = 2.86).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoresheet.xlsx
+++ b/scoresheet.xlsx
@@ -627,6 +627,9 @@
           <t>B3 Atalanta</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -634,6 +637,9 @@
           <t>B3 Ipswich</t>
         </is>
       </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -641,6 +647,9 @@
           <t>G4 Reign</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -648,6 +657,9 @@
           <t>B4 Brentford</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -655,6 +667,9 @@
           <t>G5 Angel City</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -662,6 +677,9 @@
           <t>B5 Benfica</t>
         </is>
       </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -669,6 +687,9 @@
           <t>B5 Dortmund</t>
         </is>
       </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -676,6 +697,9 @@
           <t>B5 Napoli</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -683,6 +707,9 @@
           <t>G6 Arsenal</t>
         </is>
       </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -690,6 +717,9 @@
           <t>G6 Barcelona</t>
         </is>
       </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -697,6 +727,9 @@
           <t>G7 Ajax</t>
         </is>
       </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -704,6 +737,9 @@
           <t>G7 Chelsea</t>
         </is>
       </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -711,12 +747,18 @@
           <t>G8 Courage</t>
         </is>
       </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>G8 Pride</t>
         </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round Week 3 4.5 scores up to 5
Per the organizer's call, every 4.5 score in Week 3 rounds up to 5 so
the standings stay on whole-number totals. Updated scoresheet.xlsx,
all three apps' RESULTS, and the challenge teams' explicit awayScores.

Impact on standings (vs the fractional version):
- Angel City: 7 -> 5 pts (W vs USA becomes T at 5-5)
- Courage:    9 -> 7 pts (W vs Brentford becomes T at 5-5)
- Benfica:    6 -> 4 pts (W vs Napoli becomes T at 5-5 — wait, that
                          was 5-4.5; now 5-5 = T)
- Brentford:  3 -> 4 pts (gains a draw from the Courage match)
- Ipswich, Reign, Atalanta, Pride, Arsenal, Ajax, Dortmund, Barcelona,
  Chelsea, Napoli, Mexico — unchanged

QF lineup unchanged: Angel City + Ipswich, Arsenal + Ajax,
Pride + Atalanta, Courage + Benfica (Benfica wins the Group D
runner-up spot on the GF tiebreaker, 13 vs Brentford's 11).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoresheet.xlsx
+++ b/scoresheet.xlsx
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Process Week 4 results (May 18) — Quarterfinals + Scoring Title
Quarterfinal results (all four higher seeds won):
- QF1: France (Angel City)  5 - 3 Netherlands (Ajax)
- QF2: Brazil (Pride)        4 - 3 Portugal (Benfica)
- QF3: Spain (Arsenal)       5 - 4 Morocco (Ipswich)
- QF4: Colombia (Courage)    5 - 4 Croatia (Atalanta)

Semifinal matchups (added to SCHEDULE[5] and BRACKET.sf):
- SF1: France vs Brazil
- SF2: Spain vs Colombia

Scoring Title (Week 4): recorded each team's quiz-only goals (no
tik-tok bonus, since the head-to-head only resolves bracket matches).
Tally per team ranges 2-4 across all 14 BSC sides.

Bumped CURRENT_WEEK to 5 in player + admin apps. Coach app stays at
Week 4 until Week 5 trivia content is provided. Added week 4 tab to
scoresheet.xlsx with the scoring-title view of goals.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoresheet.xlsx
+++ b/scoresheet.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="week 1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="week 2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="week 3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="week 4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -926,4 +927,165 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Goals</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B3 Atalanta</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B3 Ipswich</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>G4 Reign</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B4 Brentford</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>G5 Angel City</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B5 Benfica</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B5 Dortmund</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B5 Napoli</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>G6 Arsenal</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>G6 Barcelona</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>G7 Ajax</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>G7 Chelsea</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>G8 Courage</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>G8 Pride</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Week 4 Scoring Title — apply +1 bonus for tik toks above league avg
Correction from the organizer: Week 4 Scoring Title goals are quiz
answers correct PLUS one bonus goal for any team whose tik toks
beat the league average of 149.5.

Teams that got the +1 bonus (over 149.5 tik toks):
- Angel City  4 -> 5 (177 tt)
- Arsenal     4 -> 5 (203 tt)
- Courage     4 -> 5 (211 tt)
- Barcelona   3 -> 4 (207 tt)
- Ajax        3 -> 4 (151 tt)
- Pride       3 -> 4 (248 tt)

Teams unchanged (below avg or non-submitter avg fill):
Atalanta, Ipswich, Brentford (each 4); Chelsea, Benfica, Dortmund,
Napoli (each 3); Reign (2).

Updated scoresheet.xlsx week 4 tab and SCORING_TITLE[4] in all three
apps.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scoresheet.xlsx
+++ b/scoresheet.xlsx
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1072,7 +1072,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>